<commit_message>
Actualización tareas y modificación de preguntas para la entrevista con la bibliotecaria
</commit_message>
<xml_diff>
--- a/Tareas.xlsx
+++ b/Tareas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julia_4m9iwa1\Desktop\Julián\IUSH\Investigación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E2CDBAE-46C2-48D3-ABEA-3B2FFB1307DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B79235A5-82D9-493B-8B9D-92214B12F541}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -431,7 +431,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -445,9 +445,6 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -456,18 +453,6 @@
     </xf>
     <xf numFmtId="14" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -524,6 +509,15 @@
     <xf numFmtId="14" fontId="1" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -540,6 +534,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -869,95 +866,95 @@
   <sheetData>
     <row r="1" spans="2:25" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="2:25" x14ac:dyDescent="0.35">
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="28"/>
-      <c r="K2" s="28"/>
-      <c r="L2" s="28"/>
-      <c r="M2" s="28"/>
-      <c r="N2" s="28"/>
-      <c r="O2" s="28"/>
-      <c r="P2" s="28"/>
-      <c r="Q2" s="28"/>
-      <c r="R2" s="28"/>
-      <c r="S2" s="28"/>
-      <c r="T2" s="28"/>
-      <c r="U2" s="28"/>
-      <c r="V2" s="28"/>
-      <c r="W2" s="28"/>
-      <c r="X2" s="28"/>
-      <c r="Y2" s="29"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="26"/>
+      <c r="M2" s="26"/>
+      <c r="N2" s="26"/>
+      <c r="O2" s="26"/>
+      <c r="P2" s="26"/>
+      <c r="Q2" s="26"/>
+      <c r="R2" s="26"/>
+      <c r="S2" s="26"/>
+      <c r="T2" s="26"/>
+      <c r="U2" s="26"/>
+      <c r="V2" s="26"/>
+      <c r="W2" s="26"/>
+      <c r="X2" s="26"/>
+      <c r="Y2" s="27"/>
     </row>
     <row r="3" spans="2:25" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="30"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="31"/>
-      <c r="I3" s="31"/>
-      <c r="J3" s="31"/>
-      <c r="K3" s="31"/>
-      <c r="L3" s="31"/>
-      <c r="M3" s="31"/>
-      <c r="N3" s="31"/>
-      <c r="O3" s="31"/>
-      <c r="P3" s="31"/>
-      <c r="Q3" s="31"/>
-      <c r="R3" s="31"/>
-      <c r="S3" s="31"/>
-      <c r="T3" s="31"/>
-      <c r="U3" s="31"/>
-      <c r="V3" s="31"/>
-      <c r="W3" s="31"/>
-      <c r="X3" s="31"/>
-      <c r="Y3" s="32"/>
+      <c r="B3" s="28"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+      <c r="J3" s="29"/>
+      <c r="K3" s="29"/>
+      <c r="L3" s="29"/>
+      <c r="M3" s="29"/>
+      <c r="N3" s="29"/>
+      <c r="O3" s="29"/>
+      <c r="P3" s="29"/>
+      <c r="Q3" s="29"/>
+      <c r="R3" s="29"/>
+      <c r="S3" s="29"/>
+      <c r="T3" s="29"/>
+      <c r="U3" s="29"/>
+      <c r="V3" s="29"/>
+      <c r="W3" s="29"/>
+      <c r="X3" s="29"/>
+      <c r="Y3" s="30"/>
     </row>
     <row r="4" spans="2:25" x14ac:dyDescent="0.35">
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="9" t="s">
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="I4" s="10"/>
-      <c r="J4" s="10"/>
-      <c r="K4" s="10"/>
-      <c r="L4" s="10"/>
-      <c r="M4" s="11"/>
-      <c r="N4" s="9" t="s">
+      <c r="I4" s="23"/>
+      <c r="J4" s="23"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="24"/>
+      <c r="N4" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="O4" s="10"/>
-      <c r="P4" s="10"/>
-      <c r="Q4" s="10"/>
-      <c r="R4" s="10"/>
-      <c r="S4" s="11"/>
-      <c r="T4" s="9" t="s">
+      <c r="O4" s="23"/>
+      <c r="P4" s="23"/>
+      <c r="Q4" s="23"/>
+      <c r="R4" s="23"/>
+      <c r="S4" s="24"/>
+      <c r="T4" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="U4" s="10"/>
-      <c r="V4" s="10"/>
-      <c r="W4" s="10"/>
-      <c r="X4" s="10"/>
-      <c r="Y4" s="11"/>
+      <c r="U4" s="23"/>
+      <c r="V4" s="23"/>
+      <c r="W4" s="23"/>
+      <c r="X4" s="23"/>
+      <c r="Y4" s="24"/>
     </row>
     <row r="5" spans="2:25" x14ac:dyDescent="0.35">
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="7" t="s">
         <v>12</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -972,10 +969,10 @@
       <c r="F5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="13" t="s">
+      <c r="G5" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="H5" s="12" t="s">
+      <c r="H5" s="7" t="s">
         <v>12</v>
       </c>
       <c r="I5" s="2" t="s">
@@ -990,10 +987,10 @@
       <c r="L5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="M5" s="13" t="s">
+      <c r="M5" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="N5" s="12" t="s">
+      <c r="N5" s="7" t="s">
         <v>12</v>
       </c>
       <c r="O5" s="2" t="s">
@@ -1008,10 +1005,10 @@
       <c r="R5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="S5" s="13" t="s">
+      <c r="S5" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="T5" s="12" t="s">
+      <c r="T5" s="7" t="s">
         <v>12</v>
       </c>
       <c r="U5" s="2" t="s">
@@ -1026,647 +1023,653 @@
       <c r="X5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="Y5" s="13" t="s">
+      <c r="Y5" s="8" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="6" spans="2:25" ht="39" x14ac:dyDescent="0.35">
-      <c r="B6" s="12">
+      <c r="B6" s="7">
         <v>1</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="6">
         <v>46086</v>
       </c>
       <c r="F6" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="G6" s="14">
+      <c r="G6" s="9">
         <v>46086</v>
       </c>
-      <c r="H6" s="12">
+      <c r="H6" s="7">
         <v>1</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="I6" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="J6" s="6" t="s">
+      <c r="J6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="K6" s="7">
+      <c r="K6" s="6">
         <v>46090</v>
       </c>
       <c r="L6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="M6" s="14"/>
-      <c r="N6" s="12">
+      <c r="M6" s="9"/>
+      <c r="N6" s="7">
         <v>1</v>
       </c>
-      <c r="O6" s="5"/>
-      <c r="P6" s="6"/>
-      <c r="Q6" s="7"/>
+      <c r="O6" s="4"/>
+      <c r="P6" s="5"/>
+      <c r="Q6" s="6"/>
       <c r="R6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="S6" s="14"/>
-      <c r="T6" s="12">
+      <c r="S6" s="9"/>
+      <c r="T6" s="7">
         <v>1</v>
       </c>
-      <c r="U6" s="5"/>
-      <c r="V6" s="6"/>
-      <c r="W6" s="7"/>
+      <c r="U6" s="4"/>
+      <c r="V6" s="5"/>
+      <c r="W6" s="6"/>
       <c r="X6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="Y6" s="14"/>
+      <c r="Y6" s="9"/>
     </row>
     <row r="7" spans="2:25" ht="39" x14ac:dyDescent="0.35">
-      <c r="B7" s="12">
+      <c r="B7" s="7">
         <v>2</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="6">
         <v>46085</v>
       </c>
       <c r="F7" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="G7" s="14">
+      <c r="G7" s="9">
         <v>46085</v>
       </c>
-      <c r="H7" s="12">
+      <c r="H7" s="7">
         <v>2</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="I7" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="J7" s="6" t="s">
+      <c r="J7" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="K7" s="7">
+      <c r="K7" s="6">
         <v>46090</v>
       </c>
       <c r="L7" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="M7" s="14"/>
-      <c r="N7" s="12">
+        <v>1</v>
+      </c>
+      <c r="M7" s="6">
+        <v>46090</v>
+      </c>
+      <c r="N7" s="7">
         <v>2</v>
       </c>
-      <c r="O7" s="5"/>
-      <c r="P7" s="6"/>
-      <c r="Q7" s="7"/>
+      <c r="O7" s="4"/>
+      <c r="P7" s="5"/>
+      <c r="Q7" s="6"/>
       <c r="R7" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="S7" s="14"/>
-      <c r="T7" s="12">
+      <c r="S7" s="9"/>
+      <c r="T7" s="7">
         <v>2</v>
       </c>
-      <c r="U7" s="5"/>
-      <c r="V7" s="6"/>
-      <c r="W7" s="7"/>
+      <c r="U7" s="4"/>
+      <c r="V7" s="5"/>
+      <c r="W7" s="6"/>
       <c r="X7" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="Y7" s="14"/>
+      <c r="Y7" s="9"/>
     </row>
     <row r="8" spans="2:25" ht="39" x14ac:dyDescent="0.35">
-      <c r="B8" s="12">
+      <c r="B8" s="7">
         <v>3</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="6">
         <v>46085</v>
       </c>
       <c r="F8" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="G8" s="14">
+      <c r="G8" s="9">
         <v>46085</v>
       </c>
-      <c r="H8" s="12">
+      <c r="H8" s="7">
         <v>3</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="I8" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="J8" s="6" t="s">
+      <c r="J8" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="K8" s="7">
+      <c r="K8" s="6">
         <v>46090</v>
       </c>
       <c r="L8" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="M8" s="14"/>
-      <c r="N8" s="12">
+      <c r="M8" s="9"/>
+      <c r="N8" s="7">
         <v>3</v>
       </c>
-      <c r="O8" s="5"/>
-      <c r="P8" s="6"/>
-      <c r="Q8" s="7"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="5"/>
+      <c r="Q8" s="6"/>
       <c r="R8" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="S8" s="14"/>
-      <c r="T8" s="12">
+      <c r="S8" s="9"/>
+      <c r="T8" s="7">
         <v>3</v>
       </c>
-      <c r="U8" s="5"/>
-      <c r="V8" s="6"/>
-      <c r="W8" s="7"/>
+      <c r="U8" s="4"/>
+      <c r="V8" s="5"/>
+      <c r="W8" s="6"/>
       <c r="X8" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="Y8" s="14"/>
+      <c r="Y8" s="9"/>
     </row>
     <row r="9" spans="2:25" ht="39" x14ac:dyDescent="0.35">
-      <c r="B9" s="12">
+      <c r="B9" s="7">
         <v>4</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="6">
         <v>46085</v>
       </c>
       <c r="F9" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="G9" s="14">
+      <c r="G9" s="9">
         <v>46085</v>
       </c>
-      <c r="H9" s="12">
+      <c r="H9" s="7">
         <v>4</v>
       </c>
-      <c r="I9" s="6" t="s">
+      <c r="I9" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="J9" s="6" t="s">
+      <c r="J9" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="K9" s="7">
+      <c r="K9" s="6">
         <v>46090</v>
       </c>
       <c r="L9" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="M9" s="14"/>
-      <c r="N9" s="12">
+      <c r="M9" s="9"/>
+      <c r="N9" s="7">
         <v>4</v>
       </c>
-      <c r="O9" s="5"/>
-      <c r="P9" s="6"/>
-      <c r="Q9" s="7"/>
+      <c r="O9" s="4"/>
+      <c r="P9" s="5"/>
+      <c r="Q9" s="6"/>
       <c r="R9" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="S9" s="14"/>
-      <c r="T9" s="12">
+      <c r="S9" s="9"/>
+      <c r="T9" s="7">
         <v>4</v>
       </c>
-      <c r="U9" s="5"/>
-      <c r="V9" s="6"/>
-      <c r="W9" s="7"/>
+      <c r="U9" s="4"/>
+      <c r="V9" s="5"/>
+      <c r="W9" s="6"/>
       <c r="X9" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="Y9" s="14"/>
+      <c r="Y9" s="9"/>
     </row>
     <row r="10" spans="2:25" x14ac:dyDescent="0.35">
-      <c r="B10" s="12">
+      <c r="B10" s="7">
         <v>5</v>
       </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="7"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="6"/>
       <c r="F10" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="G10" s="14"/>
-      <c r="H10" s="12">
+      <c r="G10" s="9"/>
+      <c r="H10" s="7">
         <v>5</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="I10" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="J10" s="6" t="s">
+      <c r="J10" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="K10" s="7">
+      <c r="K10" s="6">
         <v>46090</v>
       </c>
       <c r="L10" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="M10" s="14"/>
-      <c r="N10" s="12">
+        <v>1</v>
+      </c>
+      <c r="M10" s="6">
+        <v>46090</v>
+      </c>
+      <c r="N10" s="7">
         <v>5</v>
       </c>
-      <c r="O10" s="5"/>
-      <c r="P10" s="6"/>
-      <c r="Q10" s="7"/>
+      <c r="O10" s="4"/>
+      <c r="P10" s="5"/>
+      <c r="Q10" s="6"/>
       <c r="R10" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="S10" s="14"/>
-      <c r="T10" s="12">
+      <c r="S10" s="9"/>
+      <c r="T10" s="7">
         <v>5</v>
       </c>
-      <c r="U10" s="5"/>
-      <c r="V10" s="6"/>
-      <c r="W10" s="7"/>
+      <c r="U10" s="4"/>
+      <c r="V10" s="5"/>
+      <c r="W10" s="6"/>
       <c r="X10" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="Y10" s="14"/>
+      <c r="Y10" s="9"/>
     </row>
     <row r="11" spans="2:25" x14ac:dyDescent="0.35">
-      <c r="B11" s="12">
+      <c r="B11" s="7">
         <v>6</v>
       </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="7"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="6"/>
       <c r="F11" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="G11" s="14"/>
-      <c r="H11" s="12">
+      <c r="G11" s="9"/>
+      <c r="H11" s="7">
         <v>6</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="I11" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="J11" s="6" t="s">
+      <c r="J11" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="K11" s="7">
+      <c r="K11" s="6">
         <v>46090</v>
       </c>
       <c r="L11" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="M11" s="14"/>
-      <c r="N11" s="12">
+        <v>1</v>
+      </c>
+      <c r="M11" s="6">
+        <v>46090</v>
+      </c>
+      <c r="N11" s="7">
         <v>6</v>
       </c>
-      <c r="O11" s="5"/>
-      <c r="P11" s="6"/>
-      <c r="Q11" s="7"/>
+      <c r="O11" s="4"/>
+      <c r="P11" s="5"/>
+      <c r="Q11" s="6"/>
       <c r="R11" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="S11" s="14"/>
-      <c r="T11" s="12">
+      <c r="S11" s="9"/>
+      <c r="T11" s="7">
         <v>6</v>
       </c>
-      <c r="U11" s="5"/>
-      <c r="V11" s="6"/>
-      <c r="W11" s="7"/>
+      <c r="U11" s="4"/>
+      <c r="V11" s="5"/>
+      <c r="W11" s="6"/>
       <c r="X11" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="Y11" s="14"/>
+      <c r="Y11" s="9"/>
     </row>
     <row r="12" spans="2:25" ht="39" x14ac:dyDescent="0.35">
-      <c r="B12" s="12">
+      <c r="B12" s="7">
         <v>7</v>
       </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="7"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="6"/>
       <c r="F12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="G12" s="14"/>
-      <c r="H12" s="12">
+      <c r="G12" s="9"/>
+      <c r="H12" s="7">
         <v>7</v>
       </c>
-      <c r="I12" s="5" t="s">
+      <c r="I12" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="J12" s="6" t="s">
+      <c r="J12" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="K12" s="7">
+      <c r="K12" s="6">
         <v>46090</v>
       </c>
       <c r="L12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="M12" s="14"/>
-      <c r="N12" s="12">
+      <c r="M12" s="9"/>
+      <c r="N12" s="7">
         <v>7</v>
       </c>
-      <c r="O12" s="5"/>
-      <c r="P12" s="6"/>
-      <c r="Q12" s="7"/>
+      <c r="O12" s="4"/>
+      <c r="P12" s="5"/>
+      <c r="Q12" s="6"/>
       <c r="R12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="S12" s="14"/>
-      <c r="T12" s="12">
+      <c r="S12" s="9"/>
+      <c r="T12" s="7">
         <v>7</v>
       </c>
-      <c r="U12" s="5"/>
-      <c r="V12" s="6"/>
-      <c r="W12" s="7"/>
+      <c r="U12" s="4"/>
+      <c r="V12" s="5"/>
+      <c r="W12" s="6"/>
       <c r="X12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="Y12" s="14"/>
+      <c r="Y12" s="9"/>
     </row>
     <row r="13" spans="2:25" ht="39" x14ac:dyDescent="0.35">
-      <c r="B13" s="12">
+      <c r="B13" s="7">
         <v>8</v>
       </c>
-      <c r="C13" s="5"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="7"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="6"/>
       <c r="F13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="G13" s="14"/>
-      <c r="H13" s="12">
+      <c r="G13" s="9"/>
+      <c r="H13" s="7">
         <v>8</v>
       </c>
-      <c r="I13" s="5" t="s">
+      <c r="I13" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="J13" s="6" t="s">
+      <c r="J13" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="K13" s="7">
+      <c r="K13" s="6">
         <v>46090</v>
       </c>
       <c r="L13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="M13" s="14"/>
-      <c r="N13" s="12">
+      <c r="M13" s="9"/>
+      <c r="N13" s="7">
         <v>8</v>
       </c>
-      <c r="O13" s="5"/>
-      <c r="P13" s="6"/>
-      <c r="Q13" s="7"/>
+      <c r="O13" s="4"/>
+      <c r="P13" s="5"/>
+      <c r="Q13" s="6"/>
       <c r="R13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="S13" s="14"/>
-      <c r="T13" s="12">
+      <c r="S13" s="9"/>
+      <c r="T13" s="7">
         <v>8</v>
       </c>
-      <c r="U13" s="5"/>
-      <c r="V13" s="6"/>
-      <c r="W13" s="7"/>
+      <c r="U13" s="4"/>
+      <c r="V13" s="5"/>
+      <c r="W13" s="6"/>
       <c r="X13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="Y13" s="14"/>
+      <c r="Y13" s="9"/>
     </row>
     <row r="14" spans="2:25" ht="39" x14ac:dyDescent="0.35">
-      <c r="B14" s="12">
+      <c r="B14" s="7">
         <v>9</v>
       </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="7"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="6"/>
       <c r="F14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="G14" s="14"/>
-      <c r="H14" s="12">
+      <c r="G14" s="9"/>
+      <c r="H14" s="7">
         <v>9</v>
       </c>
-      <c r="I14" s="5" t="s">
+      <c r="I14" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="J14" s="6" t="s">
+      <c r="J14" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="K14" s="7">
+      <c r="K14" s="6">
         <v>46090</v>
       </c>
       <c r="L14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="M14" s="14"/>
-      <c r="N14" s="12">
+      <c r="M14" s="9"/>
+      <c r="N14" s="7">
         <v>9</v>
       </c>
-      <c r="O14" s="5"/>
-      <c r="P14" s="6"/>
-      <c r="Q14" s="7"/>
+      <c r="O14" s="4"/>
+      <c r="P14" s="5"/>
+      <c r="Q14" s="6"/>
       <c r="R14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="S14" s="14"/>
-      <c r="T14" s="12">
+      <c r="S14" s="9"/>
+      <c r="T14" s="7">
         <v>9</v>
       </c>
-      <c r="U14" s="5"/>
-      <c r="V14" s="6"/>
-      <c r="W14" s="7"/>
+      <c r="U14" s="4"/>
+      <c r="V14" s="5"/>
+      <c r="W14" s="6"/>
       <c r="X14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="Y14" s="14"/>
+      <c r="Y14" s="9"/>
     </row>
     <row r="15" spans="2:25" ht="39" x14ac:dyDescent="0.35">
-      <c r="B15" s="21">
+      <c r="B15" s="16">
         <v>10</v>
       </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="23"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="25" t="b">
-        <v>0</v>
-      </c>
-      <c r="G15" s="26"/>
-      <c r="H15" s="12">
+      <c r="C15" s="17"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="20" t="b">
+        <v>0</v>
+      </c>
+      <c r="G15" s="21"/>
+      <c r="H15" s="7">
         <v>10</v>
       </c>
-      <c r="I15" s="23" t="s">
+      <c r="I15" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="J15" s="23" t="s">
+      <c r="J15" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="K15" s="24">
+      <c r="K15" s="19">
         <v>46090</v>
       </c>
-      <c r="L15" s="25" t="b">
-        <v>0</v>
-      </c>
-      <c r="M15" s="26"/>
-      <c r="N15" s="12">
+      <c r="L15" s="20" t="b">
+        <v>0</v>
+      </c>
+      <c r="M15" s="21"/>
+      <c r="N15" s="7">
         <v>10</v>
       </c>
-      <c r="O15" s="22"/>
-      <c r="P15" s="23"/>
-      <c r="Q15" s="24"/>
-      <c r="R15" s="25" t="b">
-        <v>0</v>
-      </c>
-      <c r="S15" s="26"/>
-      <c r="T15" s="12">
+      <c r="O15" s="17"/>
+      <c r="P15" s="18"/>
+      <c r="Q15" s="19"/>
+      <c r="R15" s="20" t="b">
+        <v>0</v>
+      </c>
+      <c r="S15" s="21"/>
+      <c r="T15" s="7">
         <v>10</v>
       </c>
-      <c r="U15" s="22"/>
-      <c r="V15" s="23"/>
-      <c r="W15" s="24"/>
-      <c r="X15" s="25" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y15" s="26"/>
+      <c r="U15" s="17"/>
+      <c r="V15" s="18"/>
+      <c r="W15" s="19"/>
+      <c r="X15" s="20" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y15" s="21"/>
     </row>
     <row r="16" spans="2:25" x14ac:dyDescent="0.35">
-      <c r="B16" s="21">
+      <c r="B16" s="16">
         <v>11</v>
       </c>
-      <c r="C16" s="22"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="25" t="b">
-        <v>0</v>
-      </c>
-      <c r="G16" s="26"/>
-      <c r="H16" s="12">
+      <c r="C16" s="17"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="20" t="b">
+        <v>0</v>
+      </c>
+      <c r="G16" s="21"/>
+      <c r="H16" s="7">
         <v>11</v>
       </c>
-      <c r="I16" s="22"/>
-      <c r="J16" s="23"/>
-      <c r="K16" s="24"/>
-      <c r="L16" s="25" t="b">
-        <v>0</v>
-      </c>
-      <c r="M16" s="26"/>
-      <c r="N16" s="12">
+      <c r="I16" s="17"/>
+      <c r="J16" s="18"/>
+      <c r="K16" s="19"/>
+      <c r="L16" s="20" t="b">
+        <v>0</v>
+      </c>
+      <c r="M16" s="21"/>
+      <c r="N16" s="7">
         <v>11</v>
       </c>
-      <c r="O16" s="22"/>
-      <c r="P16" s="23"/>
-      <c r="Q16" s="24"/>
-      <c r="R16" s="25" t="b">
-        <v>0</v>
-      </c>
-      <c r="S16" s="26"/>
-      <c r="T16" s="12">
+      <c r="O16" s="17"/>
+      <c r="P16" s="18"/>
+      <c r="Q16" s="19"/>
+      <c r="R16" s="20" t="b">
+        <v>0</v>
+      </c>
+      <c r="S16" s="21"/>
+      <c r="T16" s="7">
         <v>11</v>
       </c>
-      <c r="U16" s="22"/>
-      <c r="V16" s="23"/>
-      <c r="W16" s="24"/>
-      <c r="X16" s="25" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y16" s="26"/>
+      <c r="U16" s="17"/>
+      <c r="V16" s="18"/>
+      <c r="W16" s="19"/>
+      <c r="X16" s="20" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y16" s="21"/>
     </row>
     <row r="17" spans="2:25" x14ac:dyDescent="0.35">
-      <c r="B17" s="21">
+      <c r="B17" s="16">
         <v>12</v>
       </c>
-      <c r="C17" s="22"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="25" t="b">
-        <v>0</v>
-      </c>
-      <c r="G17" s="26"/>
-      <c r="H17" s="12">
+      <c r="C17" s="17"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="20" t="b">
+        <v>0</v>
+      </c>
+      <c r="G17" s="21"/>
+      <c r="H17" s="7">
         <v>12</v>
       </c>
-      <c r="I17" s="22"/>
-      <c r="J17" s="23"/>
-      <c r="K17" s="24"/>
-      <c r="L17" s="25" t="b">
-        <v>0</v>
-      </c>
-      <c r="M17" s="26"/>
-      <c r="N17" s="12">
+      <c r="I17" s="17"/>
+      <c r="J17" s="18"/>
+      <c r="K17" s="19"/>
+      <c r="L17" s="20" t="b">
+        <v>0</v>
+      </c>
+      <c r="M17" s="21"/>
+      <c r="N17" s="7">
         <v>12</v>
       </c>
-      <c r="O17" s="22"/>
-      <c r="P17" s="23"/>
-      <c r="Q17" s="24"/>
-      <c r="R17" s="25" t="b">
-        <v>0</v>
-      </c>
-      <c r="S17" s="26"/>
-      <c r="T17" s="12">
+      <c r="O17" s="17"/>
+      <c r="P17" s="18"/>
+      <c r="Q17" s="19"/>
+      <c r="R17" s="20" t="b">
+        <v>0</v>
+      </c>
+      <c r="S17" s="21"/>
+      <c r="T17" s="7">
         <v>12</v>
       </c>
-      <c r="U17" s="22"/>
-      <c r="V17" s="23"/>
-      <c r="W17" s="24"/>
-      <c r="X17" s="25" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y17" s="26"/>
+      <c r="U17" s="17"/>
+      <c r="V17" s="18"/>
+      <c r="W17" s="19"/>
+      <c r="X17" s="20" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y17" s="21"/>
     </row>
     <row r="18" spans="2:25" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B18" s="15">
+      <c r="B18" s="10">
         <v>13</v>
       </c>
-      <c r="C18" s="16"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="19" t="b">
-        <v>0</v>
-      </c>
-      <c r="G18" s="20"/>
-      <c r="H18" s="15">
+      <c r="C18" s="11"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="G18" s="15"/>
+      <c r="H18" s="10">
         <v>13</v>
       </c>
-      <c r="I18" s="17"/>
-      <c r="J18" s="17"/>
-      <c r="K18" s="18"/>
-      <c r="L18" s="19" t="b">
-        <v>0</v>
-      </c>
-      <c r="M18" s="20"/>
-      <c r="N18" s="15">
+      <c r="I18" s="12"/>
+      <c r="J18" s="12"/>
+      <c r="K18" s="13"/>
+      <c r="L18" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="M18" s="15"/>
+      <c r="N18" s="10">
         <v>13</v>
       </c>
-      <c r="O18" s="16"/>
-      <c r="P18" s="17"/>
-      <c r="Q18" s="18"/>
-      <c r="R18" s="19" t="b">
-        <v>0</v>
-      </c>
-      <c r="S18" s="20"/>
-      <c r="T18" s="15">
+      <c r="O18" s="11"/>
+      <c r="P18" s="12"/>
+      <c r="Q18" s="13"/>
+      <c r="R18" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="S18" s="15"/>
+      <c r="T18" s="10">
         <v>13</v>
       </c>
-      <c r="U18" s="16"/>
-      <c r="V18" s="17"/>
-      <c r="W18" s="18"/>
-      <c r="X18" s="19" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y18" s="20"/>
+      <c r="U18" s="11"/>
+      <c r="V18" s="12"/>
+      <c r="W18" s="13"/>
+      <c r="X18" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y18" s="15"/>
     </row>
     <row r="19" spans="2:25" x14ac:dyDescent="0.35"/>
     <row r="20" spans="2:25" x14ac:dyDescent="0.35"/>
@@ -1726,95 +1729,95 @@
   <sheetData>
     <row r="1" spans="2:25" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:25" x14ac:dyDescent="0.35">
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-      <c r="P2" s="4"/>
-      <c r="Q2" s="4"/>
-      <c r="R2" s="4"/>
-      <c r="S2" s="4"/>
-      <c r="T2" s="4"/>
-      <c r="U2" s="4"/>
-      <c r="V2" s="4"/>
-      <c r="W2" s="4"/>
-      <c r="X2" s="4"/>
-      <c r="Y2" s="4"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="31"/>
+      <c r="O2" s="31"/>
+      <c r="P2" s="31"/>
+      <c r="Q2" s="31"/>
+      <c r="R2" s="31"/>
+      <c r="S2" s="31"/>
+      <c r="T2" s="31"/>
+      <c r="U2" s="31"/>
+      <c r="V2" s="31"/>
+      <c r="W2" s="31"/>
+      <c r="X2" s="31"/>
+      <c r="Y2" s="31"/>
     </row>
     <row r="3" spans="2:25" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
-      <c r="L3" s="8"/>
-      <c r="M3" s="8"/>
-      <c r="N3" s="8"/>
-      <c r="O3" s="8"/>
-      <c r="P3" s="8"/>
-      <c r="Q3" s="8"/>
-      <c r="R3" s="8"/>
-      <c r="S3" s="8"/>
-      <c r="T3" s="8"/>
-      <c r="U3" s="8"/>
-      <c r="V3" s="8"/>
-      <c r="W3" s="8"/>
-      <c r="X3" s="8"/>
-      <c r="Y3" s="8"/>
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="31"/>
+      <c r="L3" s="31"/>
+      <c r="M3" s="31"/>
+      <c r="N3" s="31"/>
+      <c r="O3" s="31"/>
+      <c r="P3" s="31"/>
+      <c r="Q3" s="31"/>
+      <c r="R3" s="31"/>
+      <c r="S3" s="31"/>
+      <c r="T3" s="31"/>
+      <c r="U3" s="31"/>
+      <c r="V3" s="31"/>
+      <c r="W3" s="31"/>
+      <c r="X3" s="31"/>
+      <c r="Y3" s="31"/>
     </row>
     <row r="4" spans="2:25" x14ac:dyDescent="0.35">
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="9" t="s">
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="I4" s="10"/>
-      <c r="J4" s="10"/>
-      <c r="K4" s="10"/>
-      <c r="L4" s="10"/>
-      <c r="M4" s="11"/>
-      <c r="N4" s="9" t="s">
+      <c r="I4" s="23"/>
+      <c r="J4" s="23"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="24"/>
+      <c r="N4" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="O4" s="10"/>
-      <c r="P4" s="10"/>
-      <c r="Q4" s="10"/>
-      <c r="R4" s="10"/>
-      <c r="S4" s="11"/>
-      <c r="T4" s="9" t="s">
+      <c r="O4" s="23"/>
+      <c r="P4" s="23"/>
+      <c r="Q4" s="23"/>
+      <c r="R4" s="23"/>
+      <c r="S4" s="24"/>
+      <c r="T4" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="U4" s="10"/>
-      <c r="V4" s="10"/>
-      <c r="W4" s="10"/>
-      <c r="X4" s="10"/>
-      <c r="Y4" s="11"/>
+      <c r="U4" s="23"/>
+      <c r="V4" s="23"/>
+      <c r="W4" s="23"/>
+      <c r="X4" s="23"/>
+      <c r="Y4" s="24"/>
     </row>
     <row r="5" spans="2:25" x14ac:dyDescent="0.35">
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="7" t="s">
         <v>12</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -1829,10 +1832,10 @@
       <c r="F5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="13" t="s">
+      <c r="G5" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="H5" s="12" t="s">
+      <c r="H5" s="7" t="s">
         <v>12</v>
       </c>
       <c r="I5" s="2" t="s">
@@ -1847,10 +1850,10 @@
       <c r="L5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="M5" s="13" t="s">
+      <c r="M5" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="N5" s="12" t="s">
+      <c r="N5" s="7" t="s">
         <v>12</v>
       </c>
       <c r="O5" s="2" t="s">
@@ -1865,10 +1868,10 @@
       <c r="R5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="S5" s="13" t="s">
+      <c r="S5" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="T5" s="12" t="s">
+      <c r="T5" s="7" t="s">
         <v>12</v>
       </c>
       <c r="U5" s="2" t="s">
@@ -1883,429 +1886,429 @@
       <c r="X5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="Y5" s="13" t="s">
+      <c r="Y5" s="8" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="6" spans="2:25" x14ac:dyDescent="0.35">
-      <c r="B6" s="12">
+      <c r="B6" s="7">
         <v>1</v>
       </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="7"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="6"/>
       <c r="F6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="G6" s="14"/>
-      <c r="H6" s="12">
+      <c r="G6" s="9"/>
+      <c r="H6" s="7">
         <v>1</v>
       </c>
-      <c r="I6" s="5"/>
-      <c r="J6" s="6"/>
-      <c r="K6" s="7"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="6"/>
       <c r="L6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="M6" s="14"/>
-      <c r="N6" s="12">
+      <c r="M6" s="9"/>
+      <c r="N6" s="7">
         <v>1</v>
       </c>
-      <c r="O6" s="5"/>
-      <c r="P6" s="6"/>
-      <c r="Q6" s="7"/>
+      <c r="O6" s="4"/>
+      <c r="P6" s="5"/>
+      <c r="Q6" s="6"/>
       <c r="R6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="S6" s="14"/>
-      <c r="T6" s="12">
+      <c r="S6" s="9"/>
+      <c r="T6" s="7">
         <v>1</v>
       </c>
-      <c r="U6" s="5"/>
-      <c r="V6" s="6"/>
-      <c r="W6" s="7"/>
+      <c r="U6" s="4"/>
+      <c r="V6" s="5"/>
+      <c r="W6" s="6"/>
       <c r="X6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="Y6" s="14"/>
+      <c r="Y6" s="9"/>
     </row>
     <row r="7" spans="2:25" x14ac:dyDescent="0.35">
-      <c r="B7" s="12">
+      <c r="B7" s="7">
         <v>2</v>
       </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="7"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="6"/>
       <c r="F7" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="G7" s="14"/>
-      <c r="H7" s="12">
+      <c r="G7" s="9"/>
+      <c r="H7" s="7">
         <v>2</v>
       </c>
-      <c r="I7" s="5"/>
-      <c r="J7" s="6"/>
-      <c r="K7" s="7"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="6"/>
       <c r="L7" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="M7" s="14"/>
-      <c r="N7" s="12">
+      <c r="M7" s="9"/>
+      <c r="N7" s="7">
         <v>2</v>
       </c>
-      <c r="O7" s="5"/>
-      <c r="P7" s="6"/>
-      <c r="Q7" s="7"/>
+      <c r="O7" s="4"/>
+      <c r="P7" s="5"/>
+      <c r="Q7" s="6"/>
       <c r="R7" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="S7" s="14"/>
-      <c r="T7" s="12">
+      <c r="S7" s="9"/>
+      <c r="T7" s="7">
         <v>2</v>
       </c>
-      <c r="U7" s="5"/>
-      <c r="V7" s="6"/>
-      <c r="W7" s="7"/>
+      <c r="U7" s="4"/>
+      <c r="V7" s="5"/>
+      <c r="W7" s="6"/>
       <c r="X7" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="Y7" s="14"/>
+      <c r="Y7" s="9"/>
     </row>
     <row r="8" spans="2:25" x14ac:dyDescent="0.35">
-      <c r="B8" s="12">
+      <c r="B8" s="7">
         <v>3</v>
       </c>
-      <c r="C8" s="5"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="7"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="6"/>
       <c r="F8" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="G8" s="14"/>
-      <c r="H8" s="12">
+      <c r="G8" s="9"/>
+      <c r="H8" s="7">
         <v>3</v>
       </c>
-      <c r="I8" s="5"/>
-      <c r="J8" s="6"/>
-      <c r="K8" s="7"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="6"/>
       <c r="L8" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="M8" s="14"/>
-      <c r="N8" s="12">
+      <c r="M8" s="9"/>
+      <c r="N8" s="7">
         <v>3</v>
       </c>
-      <c r="O8" s="5"/>
-      <c r="P8" s="6"/>
-      <c r="Q8" s="7"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="5"/>
+      <c r="Q8" s="6"/>
       <c r="R8" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="S8" s="14"/>
-      <c r="T8" s="12">
+      <c r="S8" s="9"/>
+      <c r="T8" s="7">
         <v>3</v>
       </c>
-      <c r="U8" s="5"/>
-      <c r="V8" s="6"/>
-      <c r="W8" s="7"/>
+      <c r="U8" s="4"/>
+      <c r="V8" s="5"/>
+      <c r="W8" s="6"/>
       <c r="X8" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="Y8" s="14"/>
+      <c r="Y8" s="9"/>
     </row>
     <row r="9" spans="2:25" x14ac:dyDescent="0.35">
-      <c r="B9" s="12">
+      <c r="B9" s="7">
         <v>4</v>
       </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="7"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="6"/>
       <c r="F9" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="G9" s="14"/>
-      <c r="H9" s="12">
+      <c r="G9" s="9"/>
+      <c r="H9" s="7">
         <v>4</v>
       </c>
-      <c r="I9" s="5"/>
-      <c r="J9" s="6"/>
-      <c r="K9" s="7"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="6"/>
       <c r="L9" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="M9" s="14"/>
-      <c r="N9" s="12">
+      <c r="M9" s="9"/>
+      <c r="N9" s="7">
         <v>4</v>
       </c>
-      <c r="O9" s="5"/>
-      <c r="P9" s="6"/>
-      <c r="Q9" s="7"/>
+      <c r="O9" s="4"/>
+      <c r="P9" s="5"/>
+      <c r="Q9" s="6"/>
       <c r="R9" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="S9" s="14"/>
-      <c r="T9" s="12">
+      <c r="S9" s="9"/>
+      <c r="T9" s="7">
         <v>4</v>
       </c>
-      <c r="U9" s="5"/>
-      <c r="V9" s="6"/>
-      <c r="W9" s="7"/>
+      <c r="U9" s="4"/>
+      <c r="V9" s="5"/>
+      <c r="W9" s="6"/>
       <c r="X9" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="Y9" s="14"/>
+      <c r="Y9" s="9"/>
     </row>
     <row r="10" spans="2:25" x14ac:dyDescent="0.35">
-      <c r="B10" s="12">
+      <c r="B10" s="7">
         <v>5</v>
       </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="7"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="6"/>
       <c r="F10" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="G10" s="14"/>
-      <c r="H10" s="12">
+      <c r="G10" s="9"/>
+      <c r="H10" s="7">
         <v>5</v>
       </c>
-      <c r="I10" s="5"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="7"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="6"/>
       <c r="L10" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="M10" s="14"/>
-      <c r="N10" s="12">
+      <c r="M10" s="9"/>
+      <c r="N10" s="7">
         <v>5</v>
       </c>
-      <c r="O10" s="5"/>
-      <c r="P10" s="6"/>
-      <c r="Q10" s="7"/>
+      <c r="O10" s="4"/>
+      <c r="P10" s="5"/>
+      <c r="Q10" s="6"/>
       <c r="R10" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="S10" s="14"/>
-      <c r="T10" s="12">
+      <c r="S10" s="9"/>
+      <c r="T10" s="7">
         <v>5</v>
       </c>
-      <c r="U10" s="5"/>
-      <c r="V10" s="6"/>
-      <c r="W10" s="7"/>
+      <c r="U10" s="4"/>
+      <c r="V10" s="5"/>
+      <c r="W10" s="6"/>
       <c r="X10" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="Y10" s="14"/>
+      <c r="Y10" s="9"/>
     </row>
     <row r="11" spans="2:25" x14ac:dyDescent="0.35">
-      <c r="B11" s="12">
+      <c r="B11" s="7">
         <v>6</v>
       </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="7"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="6"/>
       <c r="F11" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="G11" s="14"/>
-      <c r="H11" s="12">
+      <c r="G11" s="9"/>
+      <c r="H11" s="7">
         <v>6</v>
       </c>
-      <c r="I11" s="5"/>
-      <c r="J11" s="6"/>
-      <c r="K11" s="7"/>
+      <c r="I11" s="4"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="6"/>
       <c r="L11" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="M11" s="14"/>
-      <c r="N11" s="12">
+      <c r="M11" s="9"/>
+      <c r="N11" s="7">
         <v>6</v>
       </c>
-      <c r="O11" s="5"/>
-      <c r="P11" s="6"/>
-      <c r="Q11" s="7"/>
+      <c r="O11" s="4"/>
+      <c r="P11" s="5"/>
+      <c r="Q11" s="6"/>
       <c r="R11" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="S11" s="14"/>
-      <c r="T11" s="12">
+      <c r="S11" s="9"/>
+      <c r="T11" s="7">
         <v>6</v>
       </c>
-      <c r="U11" s="5"/>
-      <c r="V11" s="6"/>
-      <c r="W11" s="7"/>
+      <c r="U11" s="4"/>
+      <c r="V11" s="5"/>
+      <c r="W11" s="6"/>
       <c r="X11" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="Y11" s="14"/>
+      <c r="Y11" s="9"/>
     </row>
     <row r="12" spans="2:25" x14ac:dyDescent="0.35">
-      <c r="B12" s="12">
+      <c r="B12" s="7">
         <v>7</v>
       </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="7"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="6"/>
       <c r="F12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="G12" s="14"/>
-      <c r="H12" s="12">
+      <c r="G12" s="9"/>
+      <c r="H12" s="7">
         <v>7</v>
       </c>
-      <c r="I12" s="5"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="7"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="6"/>
       <c r="L12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="M12" s="14"/>
-      <c r="N12" s="12">
+      <c r="M12" s="9"/>
+      <c r="N12" s="7">
         <v>7</v>
       </c>
-      <c r="O12" s="5"/>
-      <c r="P12" s="6"/>
-      <c r="Q12" s="7"/>
+      <c r="O12" s="4"/>
+      <c r="P12" s="5"/>
+      <c r="Q12" s="6"/>
       <c r="R12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="S12" s="14"/>
-      <c r="T12" s="12">
+      <c r="S12" s="9"/>
+      <c r="T12" s="7">
         <v>7</v>
       </c>
-      <c r="U12" s="5"/>
-      <c r="V12" s="6"/>
-      <c r="W12" s="7"/>
+      <c r="U12" s="4"/>
+      <c r="V12" s="5"/>
+      <c r="W12" s="6"/>
       <c r="X12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="Y12" s="14"/>
+      <c r="Y12" s="9"/>
     </row>
     <row r="13" spans="2:25" x14ac:dyDescent="0.35">
-      <c r="B13" s="12">
+      <c r="B13" s="7">
         <v>8</v>
       </c>
-      <c r="C13" s="5"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="7"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="6"/>
       <c r="F13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="G13" s="14"/>
-      <c r="H13" s="12">
+      <c r="G13" s="9"/>
+      <c r="H13" s="7">
         <v>8</v>
       </c>
-      <c r="I13" s="5"/>
-      <c r="J13" s="6"/>
-      <c r="K13" s="7"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="6"/>
       <c r="L13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="M13" s="14"/>
-      <c r="N13" s="12">
+      <c r="M13" s="9"/>
+      <c r="N13" s="7">
         <v>8</v>
       </c>
-      <c r="O13" s="5"/>
-      <c r="P13" s="6"/>
-      <c r="Q13" s="7"/>
+      <c r="O13" s="4"/>
+      <c r="P13" s="5"/>
+      <c r="Q13" s="6"/>
       <c r="R13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="S13" s="14"/>
-      <c r="T13" s="12">
+      <c r="S13" s="9"/>
+      <c r="T13" s="7">
         <v>8</v>
       </c>
-      <c r="U13" s="5"/>
-      <c r="V13" s="6"/>
-      <c r="W13" s="7"/>
+      <c r="U13" s="4"/>
+      <c r="V13" s="5"/>
+      <c r="W13" s="6"/>
       <c r="X13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="Y13" s="14"/>
+      <c r="Y13" s="9"/>
     </row>
     <row r="14" spans="2:25" x14ac:dyDescent="0.35">
-      <c r="B14" s="12">
+      <c r="B14" s="7">
         <v>9</v>
       </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="7"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="6"/>
       <c r="F14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="G14" s="14"/>
-      <c r="H14" s="12">
+      <c r="G14" s="9"/>
+      <c r="H14" s="7">
         <v>9</v>
       </c>
-      <c r="I14" s="5"/>
-      <c r="J14" s="6"/>
-      <c r="K14" s="7"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="6"/>
       <c r="L14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="M14" s="14"/>
-      <c r="N14" s="12">
+      <c r="M14" s="9"/>
+      <c r="N14" s="7">
         <v>9</v>
       </c>
-      <c r="O14" s="5"/>
-      <c r="P14" s="6"/>
-      <c r="Q14" s="7"/>
+      <c r="O14" s="4"/>
+      <c r="P14" s="5"/>
+      <c r="Q14" s="6"/>
       <c r="R14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="S14" s="14"/>
-      <c r="T14" s="12">
+      <c r="S14" s="9"/>
+      <c r="T14" s="7">
         <v>9</v>
       </c>
-      <c r="U14" s="5"/>
-      <c r="V14" s="6"/>
-      <c r="W14" s="7"/>
+      <c r="U14" s="4"/>
+      <c r="V14" s="5"/>
+      <c r="W14" s="6"/>
       <c r="X14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="Y14" s="14"/>
+      <c r="Y14" s="9"/>
     </row>
     <row r="15" spans="2:25" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B15" s="15">
+      <c r="B15" s="10">
         <v>10</v>
       </c>
-      <c r="C15" s="16"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="19" t="b">
-        <v>0</v>
-      </c>
-      <c r="G15" s="20"/>
-      <c r="H15" s="15">
+      <c r="C15" s="11"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="G15" s="15"/>
+      <c r="H15" s="10">
         <v>10</v>
       </c>
-      <c r="I15" s="16"/>
-      <c r="J15" s="17"/>
-      <c r="K15" s="18"/>
-      <c r="L15" s="19" t="b">
-        <v>0</v>
-      </c>
-      <c r="M15" s="20"/>
-      <c r="N15" s="15">
+      <c r="I15" s="11"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="13"/>
+      <c r="L15" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="M15" s="15"/>
+      <c r="N15" s="10">
         <v>10</v>
       </c>
-      <c r="O15" s="16"/>
-      <c r="P15" s="17"/>
-      <c r="Q15" s="18"/>
-      <c r="R15" s="19" t="b">
-        <v>0</v>
-      </c>
-      <c r="S15" s="20"/>
-      <c r="T15" s="15">
+      <c r="O15" s="11"/>
+      <c r="P15" s="12"/>
+      <c r="Q15" s="13"/>
+      <c r="R15" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="S15" s="15"/>
+      <c r="T15" s="10">
         <v>10</v>
       </c>
-      <c r="U15" s="16"/>
-      <c r="V15" s="17"/>
-      <c r="W15" s="18"/>
-      <c r="X15" s="19" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y15" s="20"/>
+      <c r="U15" s="11"/>
+      <c r="V15" s="12"/>
+      <c r="W15" s="13"/>
+      <c r="X15" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y15" s="15"/>
     </row>
     <row r="16" spans="2:25" x14ac:dyDescent="0.35"/>
     <row r="17" x14ac:dyDescent="0.35"/>

</xml_diff>

<commit_message>
Se adjuntaron las encuestas
</commit_message>
<xml_diff>
--- a/Tareas.xlsx
+++ b/Tareas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julia_4m9iwa1\Desktop\Julián\IUSH\Investigación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B79235A5-82D9-493B-8B9D-92214B12F541}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FD8907B-2AA2-4D0E-818E-43019F6DAC03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1229,9 +1229,11 @@
         <v>46090</v>
       </c>
       <c r="L9" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="M9" s="9"/>
+        <v>1</v>
+      </c>
+      <c r="M9" s="9">
+        <v>46092</v>
+      </c>
       <c r="N9" s="7">
         <v>4</v>
       </c>

</xml_diff>

<commit_message>
Se actualizan tareas, se comparte archivo de enlaces importantes y se crea el formato de visitas para validar con los asesores
</commit_message>
<xml_diff>
--- a/Tareas.xlsx
+++ b/Tareas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julia_4m9iwa1\Desktop\Julián\IUSH\Investigación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B24401E-102A-4247-BB8D-542424B5C6EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4E31F96-999C-449A-9526-DB856737652B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1225,9 +1225,11 @@
         <v>46095</v>
       </c>
       <c r="R8" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="S8" s="9"/>
+        <v>1</v>
+      </c>
+      <c r="S8" s="9">
+        <v>46099</v>
+      </c>
       <c r="T8" s="7">
         <v>3</v>
       </c>
@@ -1345,9 +1347,11 @@
         <v>46095</v>
       </c>
       <c r="R10" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="S10" s="9"/>
+        <v>1</v>
+      </c>
+      <c r="S10" s="9">
+        <v>46097</v>
+      </c>
       <c r="T10" s="7">
         <v>5</v>
       </c>
@@ -1513,9 +1517,11 @@
         <v>46095</v>
       </c>
       <c r="R13" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="S13" s="9"/>
+        <v>1</v>
+      </c>
+      <c r="S13" s="9">
+        <v>46099</v>
+      </c>
       <c r="T13" s="7">
         <v>8</v>
       </c>

</xml_diff>